<commit_message>
Add regional and transit samples to October timeliness sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BvLRvWFQaEyTcRGBj2ZeMz
</commit_message>
<xml_diff>
--- a/時效抽測/抽測國內快捷時效_115年.xlsx
+++ b/時效抽測/抽測國內快捷時效_115年.xlsx
@@ -1113,7 +1113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="117">
   <si>
     <t xml:space="preserve">中和郵局  抽測國內快捷情形報告單</t>
   </si>
@@ -1355,48 +1355,7 @@
     <t xml:space="preserve">符合時效比例</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">平均               </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">數</t>
-    </r>
+    <t xml:space="preserve">平均               (時)數</t>
   </si>
   <si>
     <t xml:space="preserve">本收本投</t>
@@ -1405,40 +1364,7 @@
     <t xml:space="preserve">主要都市間互寄</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">區域內互寄           </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">北北基、台中、高雄、中彰投地區</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">區域內互寄           (北北基、台中、高雄、中彰投地區)</t>
   </si>
   <si>
     <t xml:space="preserve">其他轉口</t>
@@ -1447,653 +1373,25 @@
     <t xml:space="preserve">說明：</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">為瞭解國內快捷郵件寄遞時效，各局快捷單位應透過</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">MQ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">或本公司全球資訊網查詢系統抽測「本收本投」、「主要都市互寄」、「區域內互寄」、「其他轉口」</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">類，每月至少各</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">件（抽查紀錄列印或記錄郵件號碼留局備查，保存</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">年），抽測結果於次月</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日前寄管轄郵局郵務科彙整，於</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日前上傳主機。</t>
-    </r>
+    <t xml:space="preserve">為瞭解國內快捷郵件寄遞時效，各局快捷單位應透過MQ或本公司全球資訊網查詢系統抽測「本收本投」、「主要都市互寄」、「區域內互寄」、「其他轉口」4類，每月至少各10件（抽查紀錄列印或記錄郵件號碼留局備查，保存1年），抽測結果於次月5日前寄管轄郵局郵務科彙整，於8日前上傳主機。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">抽測樣本：本收本投以</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時前交寄、主要都市互寄</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">11</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時前交寄、區域間互寄</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">13</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時前交寄之郵件抽測為主。</t>
-    </r>
+    <t xml:space="preserve">抽測樣本：本收本投以15時前交寄、主要都市互寄11時前交寄、區域間互寄13時前交寄之郵件抽測為主。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">寄遞時效：自「交寄郵件」到「郵件投遞中」之處理狀態時間計算，四小時以內者填「ｊ＋</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時」欄；逾四小時不逾六小時者填「ｊ＋</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時」欄，餘類推。抽測結果有不符合時效標準者，請將相關地名列出，並檢討改善。</t>
-    </r>
+    <t xml:space="preserve">寄遞時效：自「交寄郵件」到「郵件投遞中」之處理狀態時間計算，四小時以內者填「ｊ＋4時」欄；逾四小時不逾六小時者填「ｊ＋6時」欄，餘類推。抽測結果有不符合時效標準者，請將相關地名列出，並檢討改善。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">十大都市互寄係指台北市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(100-110)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、板橋市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(220)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、桃園市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(330)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、中壢市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">含平鎮，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">320</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">324)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、新竹市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(300)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、台中市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(400-408)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、彰化市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(500)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、嘉義市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(600)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、台南市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(700-709)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、高雄市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(800-804</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">806</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">807)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">互寄者。該欄位僅由該十大都市互寄局就相關之郵件抽測情形填註。</t>
-    </r>
+    <t xml:space="preserve">十大都市互寄係指台北市(100-110)、板橋市(220)、桃園市(330)、中壢市(含平鎮，320、324)、新竹市(300)、台中市(400-408)、彰化市(500)、嘉義市(600)、台南市(700-709)、高雄市(800-804、806、807)互寄者。該欄位僅由該十大都市互寄局就相關之郵件抽測情形填註。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">平均</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">數：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">((J+2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">小時投遞率</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)*2+(J+4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">小時投遞率</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)*4+(J+6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">小時投遞率</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)*6+(J+8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">小時投遞率</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)*8+(J+8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">小時以上投遞率</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)*8)/100</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。</t>
-    </r>
+    <t xml:space="preserve">平均(時)數：((J+2小時投遞率)*2+(J+4小時投遞率)*4+(J+6小時投遞率)*6+(J+8小時投遞率)*8+(J+8小時以上投遞率)*8)/100。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">製表</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">:</t>
-    </r>
+    <t xml:space="preserve">製表:</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">主管</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">:</t>
-    </r>
+    <t xml:space="preserve">主管:</t>
   </si>
   <si>
     <t xml:space="preserve">郵件號碼</t>
@@ -2111,731 +1409,23 @@
     <t xml:space="preserve">時效</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">本地互寄</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">:( 15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時前交寄之郵件</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">板橋市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">22071~81</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">92</t>
-    </r>
+    <t xml:space="preserve">本地互寄:( 15時前交寄之郵件)
+板橋市22071~81、92</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">  製表</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">:</t>
-    </r>
+    <t xml:space="preserve">  製表:</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">十大都市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">:( 11</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時前交寄之郵件</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">台北市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(100-110)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、基隆市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(200~206)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、桃園市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(330)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、中壢市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">含平鎮，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">320</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">324)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、台中市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(400-408)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、彰化市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(500)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、嘉義市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(600)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、台南市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(700-709)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、高雄市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(800-804</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">806</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">807)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">互寄者。</t>
-    </r>
+    <t xml:space="preserve">十大都市:( 11時前交寄之郵件)
+台北市(100-110)、基隆市(200~206)、桃園市(330)、中壢市(含平鎮，320、324)、台中市(400-408)、彰化市(500)、嘉義市(600)、台南市(700-709)、高雄市(800-804、806、807)互寄者。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">區域互寄</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">:( 13</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時前交寄之郵件</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)
-220</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">241</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">360</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">420</t>
-    </r>
+    <t xml:space="preserve">區域互寄:( 13時前交寄之郵件)
+220、241、360、420</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">十大都市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">:( 11</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時前交寄之郵件</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">台北市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(100-110)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、板橋市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(220)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、桃園市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(330)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、中壢市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">含平鎮，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">320</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">324)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、新竹市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(300)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、台中市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(400-408)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、彰化市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(500)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、嘉義市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(600)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、台南市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(700-709)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、高雄市</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(800-804</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">806</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">807)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">互寄者。</t>
-    </r>
+    <t xml:space="preserve">十大都市:( 11時前交寄之郵件)
+台北市(100-110)、板橋市(220)、桃園市(330)、中壢市(含平鎮，320、324)、新竹市(300)、台中市(400-408)、彰化市(500)、嘉義市(600)、台南市(700-709)、高雄市(800-804、806、807)互寄者。</t>
   </si>
   <si>
     <r>
@@ -3174,6 +1764,12 @@
     <t xml:space="preserve">90945720000850235007</t>
   </si>
   <si>
+    <t xml:space="preserve">91465822001750235004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98535124102750235006</t>
+  </si>
+  <si>
     <t xml:space="preserve">96630310018450235002</t>
   </si>
   <si>
@@ -3196,6 +1792,12 @@
   </si>
   <si>
     <t xml:space="preserve">98055832045050235008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90588832002350235009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93879780000650235006</t>
   </si>
   <si>
     <r>
@@ -3250,7 +1852,7 @@
     <numFmt numFmtId="170" formatCode="[&lt;1]hh:mm;m/d\ hh:mm"/>
     <numFmt numFmtId="171" formatCode="[h]:mm;&quot;錯誤&quot;"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="12"/>
       <name val="新細明體"/>
@@ -3282,6 +1884,7 @@
       <sz val="24"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="24"/>
@@ -3310,6 +1913,13 @@
       <sz val="16"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -3332,6 +1942,7 @@
       <sz val="14"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -3348,12 +1959,14 @@
       <sz val="18"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="16"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -3457,7 +2070,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3537,23 +2150,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3581,15 +2194,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3613,11 +2226,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4601,7 +3214,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -4840,7 +3453,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -5079,7 +3692,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -5318,7 +3931,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -6082,7 +4695,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -6321,7 +4934,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -6560,7 +5173,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -6799,7 +5412,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -7564,7 +6177,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -7803,7 +6416,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -8042,7 +6655,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -8281,7 +6894,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -9045,7 +7658,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -9284,7 +7897,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -9523,7 +8136,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -9762,7 +8375,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -10586,7 +9199,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -10885,7 +9498,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -11184,7 +9797,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -11483,7 +10096,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -11727,54 +10340,54 @@
       <c r="B6" s="18"/>
       <c r="C6" s="13" t="n">
         <f aca="false">D6+F6+H6+J6+L6</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"J+2")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="15" t="str">
+      <c r="E6" s="15" t="n">
         <f aca="false">IF($C6=0,"",D6/$C6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"J+4")</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="G6" s="15" t="n">
         <f aca="false">IF($C6=0,"",F6/$C6)</f>
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="H6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"J+6")</f>
-        <v>0</v>
-      </c>
-      <c r="I6" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="I6" s="15" t="n">
         <f aca="false">IF($C6=0,"",H6/$C6)</f>
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="J6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"J+8")</f>
         <v>0</v>
       </c>
-      <c r="K6" s="15" t="str">
+      <c r="K6" s="15" t="n">
         <f aca="false">IF($C6=0,"",J6/$C6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"8以上")</f>
         <v>0</v>
       </c>
-      <c r="M6" s="15" t="str">
+      <c r="M6" s="15" t="n">
         <f aca="false">IF($C6=0,"",L6/$C6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N6" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="17" t="str">
+      <c r="O6" s="17" t="n">
         <f aca="false">IF($C6=0,"",(D6*2+F6*4+H6*6+J6*8+L6*8)/$C6)</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11784,7 +10397,7 @@
       <c r="B7" s="19"/>
       <c r="C7" s="13" t="n">
         <f aca="false">D7+F7+H7+J7+L7</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D7" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$63:$E$77,"J+2")</f>
@@ -11808,15 +10421,15 @@
       </c>
       <c r="I7" s="15" t="n">
         <f aca="false">IF($C7=0,"",H7/$C7)</f>
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="J7" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$63:$E$77,"J+8")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K7" s="15" t="n">
         <f aca="false">IF($C7=0,"",J7/$C7)</f>
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="L7" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$63:$E$77,"8以上")</f>
@@ -11831,7 +10444,7 @@
       </c>
       <c r="O7" s="17" t="n">
         <f aca="false">IF($C7=0,"",(D7*2+F7*4+H7*6+J7*8+L7*8)/$C7)</f>
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12247,7 +10860,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -12486,7 +11099,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -12725,7 +11338,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -12964,7 +11577,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -13244,7 +11857,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -13573,7 +12186,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -13609,29 +12222,41 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="35"/>
-      <c r="B43" s="36"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="38" t="str">
+      <c r="A43" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="B43" s="36" t="n">
+        <v>46296.3951388889</v>
+      </c>
+      <c r="C43" s="37" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D43" s="38" t="n">
         <f aca="false">IF(OR(B43="",C43=""),"",ROUND((IF(C43&lt;1,INT(B43)+C43,C43)-B43)*1440,0)/1440)</f>
-        <v/>
+        <v>0.154861111111111</v>
       </c>
       <c r="E43" s="39" t="str">
         <f aca="false">IF(D43="","",IF(D43&lt;0,"打日期",IF(D43*1440&lt;=120,"J+2",IF(D43*1440&lt;=240,"J+4",IF(D43*1440&lt;=360,"J+6",IF(D43*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+4</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="35"/>
-      <c r="B44" s="36"/>
-      <c r="C44" s="37"/>
-      <c r="D44" s="38" t="str">
+      <c r="A44" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="36" t="n">
+        <v>46296.4673611111</v>
+      </c>
+      <c r="C44" s="37" t="n">
+        <v>0.670138888888889</v>
+      </c>
+      <c r="D44" s="38" t="n">
         <f aca="false">IF(OR(B44="",C44=""),"",ROUND((IF(C44&lt;1,INT(B44)+C44,C44)-B44)*1440,0)/1440)</f>
-        <v/>
+        <v>0.202777777777778</v>
       </c>
       <c r="E44" s="39" t="str">
         <f aca="false">IF(D44="","",IF(D44&lt;0,"打日期",IF(D44*1440&lt;=120,"J+2",IF(D44*1440&lt;=240,"J+4",IF(D44*1440&lt;=360,"J+6",IF(D44*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13812,7 +12437,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -13849,7 +12474,7 @@
     </row>
     <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="35" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B63" s="36" t="n">
         <v>46300.3569444444</v>
@@ -13868,7 +12493,7 @@
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="35" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B64" s="36" t="n">
         <v>46300.3743055556</v>
@@ -13887,7 +12512,7 @@
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="35" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B65" s="36" t="n">
         <v>46300.3958333333</v>
@@ -13906,7 +12531,7 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="35" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B66" s="36" t="n">
         <v>46300.3972222222</v>
@@ -13925,7 +12550,7 @@
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="35" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B67" s="36" t="n">
         <v>46300.4173611111</v>
@@ -13944,7 +12569,7 @@
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="35" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B68" s="36" t="n">
         <v>46300.4173611111</v>
@@ -13963,7 +12588,7 @@
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="35" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B69" s="36" t="n">
         <v>46300.4368055556</v>
@@ -13982,7 +12607,7 @@
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="35" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B70" s="36" t="n">
         <v>46300.4479166667</v>
@@ -14000,29 +12625,41 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="35"/>
-      <c r="B71" s="36"/>
-      <c r="C71" s="37"/>
-      <c r="D71" s="38" t="str">
+      <c r="A71" s="35" t="s">
+        <v>113</v>
+      </c>
+      <c r="B71" s="36" t="n">
+        <v>46296.3618055556</v>
+      </c>
+      <c r="C71" s="37" t="n">
+        <v>0.670833333333333</v>
+      </c>
+      <c r="D71" s="38" t="n">
         <f aca="false">IF(OR(B71="",C71=""),"",ROUND((IF(C71&lt;1,INT(B71)+C71,C71)-B71)*1440,0)/1440)</f>
-        <v/>
+        <v>0.309027777777778</v>
       </c>
       <c r="E71" s="39" t="str">
         <f aca="false">IF(D71="","",IF(D71&lt;0,"打日期",IF(D71*1440&lt;=120,"J+2",IF(D71*1440&lt;=240,"J+4",IF(D71*1440&lt;=360,"J+6",IF(D71*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+8</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="35"/>
-      <c r="B72" s="36"/>
-      <c r="C72" s="37"/>
-      <c r="D72" s="38" t="str">
+      <c r="A72" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B72" s="36" t="n">
+        <v>46296.3708333333</v>
+      </c>
+      <c r="C72" s="37" t="n">
+        <v>0.670138888888889</v>
+      </c>
+      <c r="D72" s="38" t="n">
         <f aca="false">IF(OR(B72="",C72=""),"",ROUND((IF(C72&lt;1,INT(B72)+C72,C72)-B72)*1440,0)/1440)</f>
-        <v/>
+        <v>0.299305555555556</v>
       </c>
       <c r="E72" s="39" t="str">
         <f aca="false">IF(D72="","",IF(D72&lt;0,"打日期",IF(D72*1440&lt;=120,"J+2",IF(D72*1440&lt;=240,"J+4",IF(D72*1440&lt;=360,"J+6",IF(D72*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+8</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14099,7 +12736,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -14173,7 +12810,7 @@
         <v>115年</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -14863,7 +13500,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -15102,7 +13739,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -15341,7 +13978,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -15580,7 +14217,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -15654,7 +14291,7 @@
         <v>115年</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -16344,7 +14981,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -16583,7 +15220,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -16822,7 +15459,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -17061,7 +15698,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -17825,7 +16462,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -18064,7 +16701,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -18303,7 +16940,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -18542,7 +17179,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -19306,7 +17943,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -19545,7 +18182,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -19784,7 +18421,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -20023,7 +18660,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>
@@ -20787,7 +19424,7 @@
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
     </row>
-    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
         <v>35</v>
       </c>
@@ -21026,7 +19663,7 @@
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
     </row>
-    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="41" t="s">
         <v>35</v>
       </c>
@@ -21265,7 +19902,7 @@
       <c r="D58" s="40"/>
       <c r="E58" s="40"/>
     </row>
-    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="41" t="s">
         <v>35</v>
       </c>
@@ -21504,7 +20141,7 @@
       <c r="D78" s="40"/>
       <c r="E78" s="40"/>
     </row>
-    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="41" t="s">
         <v>35</v>
       </c>

</xml_diff>

<commit_message>
Add local and more regional samples to October timeliness sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BvLRvWFQaEyTcRGBj2ZeMz
</commit_message>
<xml_diff>
--- a/時效抽測/抽測國內快捷時效_115年.xlsx
+++ b/時效抽測/抽測國內快捷時效_115年.xlsx
@@ -1113,7 +1113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="127">
   <si>
     <t xml:space="preserve">中和郵局  抽測國內快捷情形報告單</t>
   </si>
@@ -1719,6 +1719,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">93363722007950235002</t>
+  </si>
+  <si>
     <t xml:space="preserve">75914310327450235003</t>
   </si>
   <si>
@@ -1767,7 +1770,34 @@
     <t xml:space="preserve">91465822001750235004</t>
   </si>
   <si>
+    <t xml:space="preserve">92315524104350235004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91838724102250235004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93031022001850235006</t>
+  </si>
+  <si>
     <t xml:space="preserve">98535124102750235006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92006224105250235002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94999322006550235003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98566022004150235006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93969436002950235007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98239622003050235007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93657522006850235008</t>
   </si>
   <si>
     <t xml:space="preserve">96630310018450235002</t>
@@ -10226,54 +10256,54 @@
       <c r="B4" s="12"/>
       <c r="C4" s="13" t="n">
         <f aca="false">D4+F4+H4+J4+L4</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"J+2")</f>
         <v>0</v>
       </c>
-      <c r="E4" s="15" t="str">
+      <c r="E4" s="15" t="n">
         <f aca="false">IF($C4=0,"",D4/$C4)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"J+4")</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="G4" s="15" t="n">
         <f aca="false">IF($C4=0,"",F4/$C4)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"J+6")</f>
         <v>0</v>
       </c>
-      <c r="I4" s="15" t="str">
+      <c r="I4" s="15" t="n">
         <f aca="false">IF($C4=0,"",H4/$C4)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"J+8")</f>
         <v>0</v>
       </c>
-      <c r="K4" s="15" t="str">
+      <c r="K4" s="15" t="n">
         <f aca="false">IF($C4=0,"",J4/$C4)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"8以上")</f>
         <v>0</v>
       </c>
-      <c r="M4" s="15" t="str">
+      <c r="M4" s="15" t="n">
         <f aca="false">IF($C4=0,"",L4/$C4)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="17" t="str">
+      <c r="O4" s="17" t="n">
         <f aca="false">IF($C4=0,"",(D4*2+F4*4+H4*6+J4*8+L4*8)/$C4)</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10340,7 +10370,7 @@
       <c r="B6" s="18"/>
       <c r="C6" s="13" t="n">
         <f aca="false">D6+F6+H6+J6+L6</f>
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"J+2")</f>
@@ -10356,23 +10386,23 @@
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">IF($C6=0,"",F6/$C6)</f>
-        <v>0.5</v>
+        <v>0.0909090909090909</v>
       </c>
       <c r="H6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"J+6")</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I6" s="15" t="n">
         <f aca="false">IF($C6=0,"",H6/$C6)</f>
-        <v>0.5</v>
+        <v>0.818181818181818</v>
       </c>
       <c r="J6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"J+8")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" s="15" t="n">
         <f aca="false">IF($C6=0,"",J6/$C6)</f>
-        <v>0</v>
+        <v>0.0909090909090909</v>
       </c>
       <c r="L6" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$43:$E$57,"8以上")</f>
@@ -10387,7 +10417,7 @@
       </c>
       <c r="O6" s="17" t="n">
         <f aca="false">IF($C6=0,"",(D6*2+F6*4+H6*6+J6*8+L6*8)/$C6)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11654,16 +11684,22 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="38" t="str">
+      <c r="A3" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="36" t="n">
+        <v>46297.40625</v>
+      </c>
+      <c r="C3" s="37" t="n">
+        <v>0.54375</v>
+      </c>
+      <c r="D3" s="38" t="n">
         <f aca="false">IF(OR(B3="",C3=""),"",ROUND((IF(C3&lt;1,INT(B3)+C3,C3)-B3)*1440,0)/1440)</f>
-        <v/>
+        <v>0.1375</v>
       </c>
       <c r="E3" s="39" t="str">
         <f aca="false">IF(D3="","",IF(D3&lt;0,"打日期",IF(D3*1440&lt;=120,"J+2",IF(D3*1440&lt;=240,"J+4",IF(D3*1440&lt;=360,"J+6",IF(D3*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11894,7 +11930,7 @@
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="35" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B23" s="36" t="n">
         <v>46296.35</v>
@@ -11913,7 +11949,7 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="35" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B24" s="36" t="n">
         <v>46300.3416666667</v>
@@ -11932,7 +11968,7 @@
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B25" s="36" t="n">
         <v>46300.3444444445</v>
@@ -11951,7 +11987,7 @@
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="35" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B26" s="36" t="n">
         <v>46300.3486111111</v>
@@ -11970,7 +12006,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="35" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B27" s="36" t="n">
         <v>46300.3493055556</v>
@@ -11989,7 +12025,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="35" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B28" s="36" t="n">
         <v>46300.3555555556</v>
@@ -12008,7 +12044,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="35" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B29" s="36" t="n">
         <v>46300.3576388889</v>
@@ -12027,7 +12063,7 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="35" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B30" s="36" t="n">
         <v>46300.3618055556</v>
@@ -12046,7 +12082,7 @@
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="35" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B31" s="36" t="n">
         <v>46300.3854166667</v>
@@ -12065,7 +12101,7 @@
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="35" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B32" s="36" t="n">
         <v>46300.3875</v>
@@ -12084,7 +12120,7 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="35" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B33" s="36" t="n">
         <v>46300.4020833333</v>
@@ -12103,7 +12139,7 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="35" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B34" s="36" t="n">
         <v>46300.4097222222</v>
@@ -12122,7 +12158,7 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="35" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B35" s="36" t="n">
         <v>46300.4229166667</v>
@@ -12141,7 +12177,7 @@
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="35" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B36" s="36" t="n">
         <v>46300.425</v>
@@ -12160,7 +12196,7 @@
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B37" s="36" t="n">
         <v>46300.4319444444</v>
@@ -12223,7 +12259,7 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="35" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B43" s="36" t="n">
         <v>46296.3951388889</v>
@@ -12242,17 +12278,17 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="35" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B44" s="36" t="n">
-        <v>46296.4673611111</v>
+        <v>46296.4256944444</v>
       </c>
       <c r="C44" s="37" t="n">
         <v>0.670138888888889</v>
       </c>
       <c r="D44" s="38" t="n">
         <f aca="false">IF(OR(B44="",C44=""),"",ROUND((IF(C44&lt;1,INT(B44)+C44,C44)-B44)*1440,0)/1440)</f>
-        <v>0.202777777777778</v>
+        <v>0.244444444444444</v>
       </c>
       <c r="E44" s="39" t="str">
         <f aca="false">IF(D44="","",IF(D44&lt;0,"打日期",IF(D44*1440&lt;=120,"J+2",IF(D44*1440&lt;=240,"J+4",IF(D44*1440&lt;=360,"J+6",IF(D44*1440&lt;=480,"J+8","8以上"))))))</f>
@@ -12260,120 +12296,174 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="35"/>
-      <c r="B45" s="36"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="38" t="str">
+      <c r="A45" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="B45" s="36" t="n">
+        <v>46296.4402777778</v>
+      </c>
+      <c r="C45" s="37" t="n">
+        <v>0.671527777777778</v>
+      </c>
+      <c r="D45" s="38" t="n">
         <f aca="false">IF(OR(B45="",C45=""),"",ROUND((IF(C45&lt;1,INT(B45)+C45,C45)-B45)*1440,0)/1440)</f>
-        <v/>
+        <v>0.23125</v>
       </c>
       <c r="E45" s="39" t="str">
         <f aca="false">IF(D45="","",IF(D45&lt;0,"打日期",IF(D45*1440&lt;=120,"J+2",IF(D45*1440&lt;=240,"J+4",IF(D45*1440&lt;=360,"J+6",IF(D45*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="35"/>
-      <c r="B46" s="36"/>
-      <c r="C46" s="37"/>
-      <c r="D46" s="38" t="str">
+      <c r="A46" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="B46" s="36" t="n">
+        <v>46296.4631944444</v>
+      </c>
+      <c r="C46" s="37" t="n">
+        <v>0.670138888888889</v>
+      </c>
+      <c r="D46" s="38" t="n">
         <f aca="false">IF(OR(B46="",C46=""),"",ROUND((IF(C46&lt;1,INT(B46)+C46,C46)-B46)*1440,0)/1440)</f>
-        <v/>
+        <v>0.206944444444444</v>
       </c>
       <c r="E46" s="39" t="str">
         <f aca="false">IF(D46="","",IF(D46&lt;0,"打日期",IF(D46*1440&lt;=120,"J+2",IF(D46*1440&lt;=240,"J+4",IF(D46*1440&lt;=360,"J+6",IF(D46*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="35"/>
-      <c r="B47" s="36"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="38" t="str">
+      <c r="A47" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="B47" s="36" t="n">
+        <v>46296.4673611111</v>
+      </c>
+      <c r="C47" s="37" t="n">
+        <v>0.670138888888889</v>
+      </c>
+      <c r="D47" s="38" t="n">
         <f aca="false">IF(OR(B47="",C47=""),"",ROUND((IF(C47&lt;1,INT(B47)+C47,C47)-B47)*1440,0)/1440)</f>
-        <v/>
+        <v>0.202777777777778</v>
       </c>
       <c r="E47" s="39" t="str">
         <f aca="false">IF(D47="","",IF(D47&lt;0,"打日期",IF(D47*1440&lt;=120,"J+2",IF(D47*1440&lt;=240,"J+4",IF(D47*1440&lt;=360,"J+6",IF(D47*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="35"/>
-      <c r="B48" s="36"/>
-      <c r="C48" s="37"/>
-      <c r="D48" s="38" t="str">
+      <c r="A48" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="B48" s="36" t="n">
+        <v>46296.4895833333</v>
+      </c>
+      <c r="C48" s="37" t="n">
+        <v>0.671527777777778</v>
+      </c>
+      <c r="D48" s="38" t="n">
         <f aca="false">IF(OR(B48="",C48=""),"",ROUND((IF(C48&lt;1,INT(B48)+C48,C48)-B48)*1440,0)/1440)</f>
-        <v/>
+        <v>0.181944444444444</v>
       </c>
       <c r="E48" s="39" t="str">
         <f aca="false">IF(D48="","",IF(D48&lt;0,"打日期",IF(D48*1440&lt;=120,"J+2",IF(D48*1440&lt;=240,"J+4",IF(D48*1440&lt;=360,"J+6",IF(D48*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="35"/>
-      <c r="B49" s="36"/>
-      <c r="C49" s="37"/>
-      <c r="D49" s="38" t="str">
+      <c r="A49" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="B49" s="36" t="n">
+        <v>46296.5</v>
+      </c>
+      <c r="C49" s="37" t="n">
+        <v>0.670833333333333</v>
+      </c>
+      <c r="D49" s="38" t="n">
         <f aca="false">IF(OR(B49="",C49=""),"",ROUND((IF(C49&lt;1,INT(B49)+C49,C49)-B49)*1440,0)/1440)</f>
-        <v/>
+        <v>0.170833333333333</v>
       </c>
       <c r="E49" s="39" t="str">
         <f aca="false">IF(D49="","",IF(D49&lt;0,"打日期",IF(D49*1440&lt;=120,"J+2",IF(D49*1440&lt;=240,"J+4",IF(D49*1440&lt;=360,"J+6",IF(D49*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="35"/>
-      <c r="B50" s="36"/>
-      <c r="C50" s="37"/>
-      <c r="D50" s="38" t="str">
+      <c r="A50" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="B50" s="36" t="n">
+        <v>46296.5</v>
+      </c>
+      <c r="C50" s="37" t="n">
+        <v>0.671527777777778</v>
+      </c>
+      <c r="D50" s="38" t="n">
         <f aca="false">IF(OR(B50="",C50=""),"",ROUND((IF(C50&lt;1,INT(B50)+C50,C50)-B50)*1440,0)/1440)</f>
-        <v/>
+        <v>0.171527777777778</v>
       </c>
       <c r="E50" s="39" t="str">
         <f aca="false">IF(D50="","",IF(D50&lt;0,"打日期",IF(D50*1440&lt;=120,"J+2",IF(D50*1440&lt;=240,"J+4",IF(D50*1440&lt;=360,"J+6",IF(D50*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="35"/>
-      <c r="B51" s="36"/>
-      <c r="C51" s="37"/>
-      <c r="D51" s="38" t="str">
+      <c r="A51" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="B51" s="36" t="n">
+        <v>46297.3659722222</v>
+      </c>
+      <c r="C51" s="37" t="n">
+        <v>0.676388888888889</v>
+      </c>
+      <c r="D51" s="38" t="n">
         <f aca="false">IF(OR(B51="",C51=""),"",ROUND((IF(C51&lt;1,INT(B51)+C51,C51)-B51)*1440,0)/1440)</f>
-        <v/>
+        <v>0.310416666666667</v>
       </c>
       <c r="E51" s="39" t="str">
         <f aca="false">IF(D51="","",IF(D51&lt;0,"打日期",IF(D51*1440&lt;=120,"J+2",IF(D51*1440&lt;=240,"J+4",IF(D51*1440&lt;=360,"J+6",IF(D51*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+8</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="35"/>
-      <c r="B52" s="36"/>
-      <c r="C52" s="37"/>
-      <c r="D52" s="38" t="str">
+      <c r="A52" s="35" t="s">
+        <v>113</v>
+      </c>
+      <c r="B52" s="36" t="n">
+        <v>46297.4506944444</v>
+      </c>
+      <c r="C52" s="37" t="n">
+        <v>0.677083333333333</v>
+      </c>
+      <c r="D52" s="38" t="n">
         <f aca="false">IF(OR(B52="",C52=""),"",ROUND((IF(C52&lt;1,INT(B52)+C52,C52)-B52)*1440,0)/1440)</f>
-        <v/>
+        <v>0.226388888888889</v>
       </c>
       <c r="E52" s="39" t="str">
         <f aca="false">IF(D52="","",IF(D52&lt;0,"打日期",IF(D52*1440&lt;=120,"J+2",IF(D52*1440&lt;=240,"J+4",IF(D52*1440&lt;=360,"J+6",IF(D52*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="35"/>
-      <c r="B53" s="36"/>
-      <c r="C53" s="37"/>
-      <c r="D53" s="38" t="str">
+      <c r="A53" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B53" s="36" t="n">
+        <v>46297.4638888889</v>
+      </c>
+      <c r="C53" s="37" t="n">
+        <v>0.675694444444445</v>
+      </c>
+      <c r="D53" s="38" t="n">
         <f aca="false">IF(OR(B53="",C53=""),"",ROUND((IF(C53&lt;1,INT(B53)+C53,C53)-B53)*1440,0)/1440)</f>
-        <v/>
+        <v>0.211805555555556</v>
       </c>
       <c r="E53" s="39" t="str">
         <f aca="false">IF(D53="","",IF(D53&lt;0,"打日期",IF(D53*1440&lt;=120,"J+2",IF(D53*1440&lt;=240,"J+4",IF(D53*1440&lt;=360,"J+6",IF(D53*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12474,7 +12564,7 @@
     </row>
     <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="35" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B63" s="36" t="n">
         <v>46300.3569444444</v>
@@ -12493,7 +12583,7 @@
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="35" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B64" s="36" t="n">
         <v>46300.3743055556</v>
@@ -12512,7 +12602,7 @@
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="35" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B65" s="36" t="n">
         <v>46300.3958333333</v>
@@ -12531,7 +12621,7 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="35" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B66" s="36" t="n">
         <v>46300.3972222222</v>
@@ -12550,7 +12640,7 @@
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="35" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B67" s="36" t="n">
         <v>46300.4173611111</v>
@@ -12569,7 +12659,7 @@
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="35" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B68" s="36" t="n">
         <v>46300.4173611111</v>
@@ -12588,7 +12678,7 @@
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="35" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="B69" s="36" t="n">
         <v>46300.4368055556</v>
@@ -12607,7 +12697,7 @@
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="35" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="B70" s="36" t="n">
         <v>46300.4479166667</v>
@@ -12626,7 +12716,7 @@
     </row>
     <row r="71" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="35" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B71" s="36" t="n">
         <v>46296.3618055556</v>
@@ -12645,7 +12735,7 @@
     </row>
     <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="35" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="B72" s="36" t="n">
         <v>46296.3708333333</v>
@@ -12810,7 +12900,7 @@
         <v>115年</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -14291,7 +14381,7 @@
         <v>115年</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="I2" s="4"/>
     </row>

</xml_diff>

<commit_message>
Add three local samples to October timeliness sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BvLRvWFQaEyTcRGBj2ZeMz
</commit_message>
<xml_diff>
--- a/時效抽測/抽測國內快捷時效_115年.xlsx
+++ b/時效抽測/抽測國內快捷時效_115年.xlsx
@@ -1113,7 +1113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="130">
   <si>
     <t xml:space="preserve">中和郵局  抽測國內快捷情形報告單</t>
   </si>
@@ -1720,6 +1720,15 @@
   </si>
   <si>
     <t xml:space="preserve">93363722007950235002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92280022007850235001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92280122007850235000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92280222007850235009</t>
   </si>
   <si>
     <t xml:space="preserve">75914310327450235003</t>
@@ -10256,7 +10265,7 @@
       <c r="B4" s="12"/>
       <c r="C4" s="13" t="n">
         <f aca="false">D4+F4+H4+J4+L4</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"J+2")</f>
@@ -10272,15 +10281,15 @@
       </c>
       <c r="G4" s="15" t="n">
         <f aca="false">IF($C4=0,"",F4/$C4)</f>
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="H4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"J+6")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I4" s="15" t="n">
         <f aca="false">IF($C4=0,"",H4/$C4)</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="J4" s="14" t="n">
         <f aca="false">COUNTIF(10子本!$E$3:$E$17,"J+8")</f>
@@ -10303,7 +10312,7 @@
       </c>
       <c r="O4" s="17" t="n">
         <f aca="false">IF($C4=0,"",(D4*2+F4*4+H4*6+J4*8+L4*8)/$C4)</f>
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11703,42 +11712,60 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="38" t="str">
+      <c r="A4" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="36" t="n">
+        <v>46300.36875</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>0.551388888888889</v>
+      </c>
+      <c r="D4" s="38" t="n">
         <f aca="false">IF(OR(B4="",C4=""),"",ROUND((IF(C4&lt;1,INT(B4)+C4,C4)-B4)*1440,0)/1440)</f>
-        <v/>
+        <v>0.182638888888889</v>
       </c>
       <c r="E4" s="39" t="str">
         <f aca="false">IF(D4="","",IF(D4&lt;0,"打日期",IF(D4*1440&lt;=120,"J+2",IF(D4*1440&lt;=240,"J+4",IF(D4*1440&lt;=360,"J+6",IF(D4*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="38" t="str">
+      <c r="A5" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="36" t="n">
+        <v>46300.36875</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>0.552083333333333</v>
+      </c>
+      <c r="D5" s="38" t="n">
         <f aca="false">IF(OR(B5="",C5=""),"",ROUND((IF(C5&lt;1,INT(B5)+C5,C5)-B5)*1440,0)/1440)</f>
-        <v/>
+        <v>0.183333333333333</v>
       </c>
       <c r="E5" s="39" t="str">
         <f aca="false">IF(D5="","",IF(D5&lt;0,"打日期",IF(D5*1440&lt;=120,"J+2",IF(D5*1440&lt;=240,"J+4",IF(D5*1440&lt;=360,"J+6",IF(D5*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="38" t="str">
+      <c r="A6" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>46300.36875</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>0.551388888888889</v>
+      </c>
+      <c r="D6" s="38" t="n">
         <f aca="false">IF(OR(B6="",C6=""),"",ROUND((IF(C6&lt;1,INT(B6)+C6,C6)-B6)*1440,0)/1440)</f>
-        <v/>
+        <v>0.182638888888889</v>
       </c>
       <c r="E6" s="39" t="str">
         <f aca="false">IF(D6="","",IF(D6&lt;0,"打日期",IF(D6*1440&lt;=120,"J+2",IF(D6*1440&lt;=240,"J+4",IF(D6*1440&lt;=360,"J+6",IF(D6*1440&lt;=480,"J+8","8以上"))))))</f>
-        <v/>
+        <v>J+6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11930,7 +11957,7 @@
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="35" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B23" s="36" t="n">
         <v>46296.35</v>
@@ -11949,7 +11976,7 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="35" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B24" s="36" t="n">
         <v>46300.3416666667</v>
@@ -11968,7 +11995,7 @@
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="35" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B25" s="36" t="n">
         <v>46300.3444444445</v>
@@ -11987,7 +12014,7 @@
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="35" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B26" s="36" t="n">
         <v>46300.3486111111</v>
@@ -12006,7 +12033,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="35" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B27" s="36" t="n">
         <v>46300.3493055556</v>
@@ -12025,7 +12052,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="35" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B28" s="36" t="n">
         <v>46300.3555555556</v>
@@ -12044,7 +12071,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="35" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B29" s="36" t="n">
         <v>46300.3576388889</v>
@@ -12063,7 +12090,7 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="35" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B30" s="36" t="n">
         <v>46300.3618055556</v>
@@ -12082,7 +12109,7 @@
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="35" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B31" s="36" t="n">
         <v>46300.3854166667</v>
@@ -12101,7 +12128,7 @@
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="35" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B32" s="36" t="n">
         <v>46300.3875</v>
@@ -12120,7 +12147,7 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="35" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B33" s="36" t="n">
         <v>46300.4020833333</v>
@@ -12139,7 +12166,7 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="35" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B34" s="36" t="n">
         <v>46300.4097222222</v>
@@ -12158,7 +12185,7 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="35" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B35" s="36" t="n">
         <v>46300.4229166667</v>
@@ -12177,7 +12204,7 @@
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="35" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B36" s="36" t="n">
         <v>46300.425</v>
@@ -12196,7 +12223,7 @@
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="35" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B37" s="36" t="n">
         <v>46300.4319444444</v>
@@ -12259,7 +12286,7 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="35" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B43" s="36" t="n">
         <v>46296.3951388889</v>
@@ -12278,7 +12305,7 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="35" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B44" s="36" t="n">
         <v>46296.4256944444</v>
@@ -12297,7 +12324,7 @@
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="35" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B45" s="36" t="n">
         <v>46296.4402777778</v>
@@ -12316,7 +12343,7 @@
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="35" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B46" s="36" t="n">
         <v>46296.4631944444</v>
@@ -12335,7 +12362,7 @@
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="35" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B47" s="36" t="n">
         <v>46296.4673611111</v>
@@ -12354,7 +12381,7 @@
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="35" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B48" s="36" t="n">
         <v>46296.4895833333</v>
@@ -12373,7 +12400,7 @@
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="35" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B49" s="36" t="n">
         <v>46296.5</v>
@@ -12392,7 +12419,7 @@
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="35" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B50" s="36" t="n">
         <v>46296.5</v>
@@ -12411,7 +12438,7 @@
     </row>
     <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="35" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B51" s="36" t="n">
         <v>46297.3659722222</v>
@@ -12430,7 +12457,7 @@
     </row>
     <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="35" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B52" s="36" t="n">
         <v>46297.4506944444</v>
@@ -12449,7 +12476,7 @@
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="35" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B53" s="36" t="n">
         <v>46297.4638888889</v>
@@ -12564,7 +12591,7 @@
     </row>
     <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="35" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B63" s="36" t="n">
         <v>46300.3569444444</v>
@@ -12583,7 +12610,7 @@
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="35" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B64" s="36" t="n">
         <v>46300.3743055556</v>
@@ -12602,7 +12629,7 @@
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="35" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B65" s="36" t="n">
         <v>46300.3958333333</v>
@@ -12621,7 +12648,7 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="35" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B66" s="36" t="n">
         <v>46300.3972222222</v>
@@ -12640,7 +12667,7 @@
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="35" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B67" s="36" t="n">
         <v>46300.4173611111</v>
@@ -12659,7 +12686,7 @@
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="35" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B68" s="36" t="n">
         <v>46300.4173611111</v>
@@ -12678,7 +12705,7 @@
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="35" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B69" s="36" t="n">
         <v>46300.4368055556</v>
@@ -12697,7 +12724,7 @@
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="35" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B70" s="36" t="n">
         <v>46300.4479166667</v>
@@ -12716,7 +12743,7 @@
     </row>
     <row r="71" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="35" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B71" s="36" t="n">
         <v>46296.3618055556</v>
@@ -12735,7 +12762,7 @@
     </row>
     <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="35" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B72" s="36" t="n">
         <v>46296.3708333333</v>
@@ -12900,7 +12927,7 @@
         <v>115年</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -14381,7 +14408,7 @@
         <v>115年</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="I2" s="4"/>
     </row>

</xml_diff>